<commit_message>
Rolodex page, 2026-10-09, Build 123
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013hSHZVu62YY9SbxQkKSbX6
</commit_message>
<xml_diff>
--- a/DFW_Rolodex.xlsx
+++ b/DFW_Rolodex.xlsx
@@ -563,7 +563,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Héctor Ibarzábal · 2026-09-30</t>
+          <t>Héctor Ibarzábal · 2026-10-09</t>
         </is>
       </c>
     </row>
@@ -32887,7 +32887,7 @@
     <row r="284">
       <c r="A284" s="14" t="inlineStr">
         <is>
-          <t>Each of the three counts reads Yes, Partly or No, with the reason in the column beside it. Yes and Partly both count as holding a count. A No does not. Holds counts how many of the three are Yes or Partly. Rolodex, Dallas-Fort Worth, 2026-09-30.</t>
+          <t>Each of the three counts reads Yes, Partly or No, with the reason in the column beside it. Yes and Partly both count as holding a count. A No does not. Holds counts how many of the three are Yes or Partly. Rolodex, Dallas-Fort Worth, 2026-10-09.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rolodex page, 2026-10-10, Build 125
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013hSHZVu62YY9SbxQkKSbX6
</commit_message>
<xml_diff>
--- a/DFW_Rolodex.xlsx
+++ b/DFW_Rolodex.xlsx
@@ -563,7 +563,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Héctor Ibarzábal · 2026-10-09</t>
+          <t>Héctor Ibarzábal · 2026-10-10</t>
         </is>
       </c>
     </row>
@@ -32887,7 +32887,7 @@
     <row r="284">
       <c r="A284" s="14" t="inlineStr">
         <is>
-          <t>Each of the three counts reads Yes, Partly or No, with the reason in the column beside it. Yes and Partly both count as holding a count. A No does not. Holds counts how many of the three are Yes or Partly. Rolodex, Dallas-Fort Worth, 2026-10-09.</t>
+          <t>Each of the three counts reads Yes, Partly or No, with the reason in the column beside it. Yes and Partly both count as holding a count. A No does not. Holds counts how many of the three are Yes or Partly. Rolodex, Dallas-Fort Worth, 2026-10-10.</t>
         </is>
       </c>
     </row>

</xml_diff>